<commit_message>
fix product qty alert for admin page
</commit_message>
<xml_diff>
--- a/trial 1(AutoRecovered).xlsx
+++ b/trial 1(AutoRecovered).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\mohamed adel work\cesar-store\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C45A995F-50EA-43A5-A903-1D4EA4C61676}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DE87C93-FD19-4816-8DC3-092BCC5D6CF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{791D22A4-40A8-4DDB-9123-A17DB6BCCBDF}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1118" uniqueCount="671">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1535" uniqueCount="676">
   <si>
     <t>active</t>
   </si>
@@ -2050,6 +2050,21 @@
   </si>
   <si>
     <t>Ceramic Fire Ashtry  (Brands)</t>
+  </si>
+  <si>
+    <t>cars-accessories</t>
+  </si>
+  <si>
+    <t>air-fresheners</t>
+  </si>
+  <si>
+    <t>additives-fluids</t>
+  </si>
+  <si>
+    <t>cars-lights</t>
+  </si>
+  <si>
+    <t>detergent</t>
   </si>
 </sst>
 </file>
@@ -2649,6 +2664,9 @@
       <c r="E2" s="5">
         <v>439.73124999999999</v>
       </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
       <c r="G2" t="s">
         <v>12</v>
       </c>
@@ -2679,6 +2697,9 @@
       <c r="E3" s="5">
         <v>238.71124999999998</v>
       </c>
+      <c r="F3">
+        <v>10</v>
+      </c>
       <c r="G3" t="s">
         <v>12</v>
       </c>
@@ -2705,6 +2726,9 @@
       <c r="E4" s="5">
         <v>1587</v>
       </c>
+      <c r="F4">
+        <v>8</v>
+      </c>
       <c r="G4" t="s">
         <v>12</v>
       </c>
@@ -2731,6 +2755,9 @@
       <c r="E5" s="5">
         <v>1851.5</v>
       </c>
+      <c r="F5">
+        <v>5</v>
+      </c>
       <c r="G5" t="s">
         <v>12</v>
       </c>
@@ -2757,6 +2784,9 @@
       <c r="E6" s="5">
         <v>1719.25</v>
       </c>
+      <c r="F6">
+        <v>15</v>
+      </c>
       <c r="G6" t="s">
         <v>12</v>
       </c>
@@ -2783,7 +2813,18 @@
       <c r="E7" s="5">
         <v>1917.625</v>
       </c>
-      <c r="H7" s="1"/>
+      <c r="F7">
+        <v>15</v>
+      </c>
+      <c r="G7" t="s">
+        <v>671</v>
+      </c>
+      <c r="H7" t="s">
+        <v>11</v>
+      </c>
+      <c r="J7" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
@@ -2801,7 +2842,18 @@
       <c r="E8" s="5">
         <v>168.61875000000001</v>
       </c>
-      <c r="H8" s="1"/>
+      <c r="F8">
+        <v>15</v>
+      </c>
+      <c r="G8" t="s">
+        <v>671</v>
+      </c>
+      <c r="H8" t="s">
+        <v>13</v>
+      </c>
+      <c r="J8" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
@@ -2819,7 +2871,18 @@
       <c r="E9" s="5">
         <v>462.875</v>
       </c>
-      <c r="H9" s="1"/>
+      <c r="F9">
+        <v>15</v>
+      </c>
+      <c r="G9" t="s">
+        <v>671</v>
+      </c>
+      <c r="H9" t="s">
+        <v>14</v>
+      </c>
+      <c r="J9" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
@@ -2837,7 +2900,18 @@
       <c r="E10" s="5">
         <v>74.721249999999998</v>
       </c>
-      <c r="H10" s="1"/>
+      <c r="F10">
+        <v>15</v>
+      </c>
+      <c r="G10" t="s">
+        <v>671</v>
+      </c>
+      <c r="H10" t="s">
+        <v>15</v>
+      </c>
+      <c r="J10" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
@@ -2855,7 +2929,18 @@
       <c r="E11" s="5">
         <v>227.47000000000003</v>
       </c>
-      <c r="H11" s="1"/>
+      <c r="F11">
+        <v>15</v>
+      </c>
+      <c r="G11" t="s">
+        <v>671</v>
+      </c>
+      <c r="H11" t="s">
+        <v>16</v>
+      </c>
+      <c r="J11" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
@@ -2873,7 +2958,18 @@
       <c r="E12" s="5">
         <v>156.61190474999998</v>
       </c>
-      <c r="H12" s="1"/>
+      <c r="F12">
+        <v>15</v>
+      </c>
+      <c r="G12" t="s">
+        <v>671</v>
+      </c>
+      <c r="H12" t="s">
+        <v>11</v>
+      </c>
+      <c r="J12" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
@@ -2891,7 +2987,18 @@
       <c r="E13" s="5">
         <v>78.027499999999989</v>
       </c>
-      <c r="H13" s="1"/>
+      <c r="F13">
+        <v>15</v>
+      </c>
+      <c r="G13" t="s">
+        <v>671</v>
+      </c>
+      <c r="H13" t="s">
+        <v>13</v>
+      </c>
+      <c r="J13" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
@@ -2909,7 +3016,18 @@
       <c r="E14" s="5">
         <v>271.11250000000001</v>
       </c>
-      <c r="H14" s="1"/>
+      <c r="F14">
+        <v>15</v>
+      </c>
+      <c r="G14" t="s">
+        <v>671</v>
+      </c>
+      <c r="H14" t="s">
+        <v>14</v>
+      </c>
+      <c r="J14" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
@@ -2927,7 +3045,18 @@
       <c r="E15" s="5">
         <v>133.41009700000001</v>
       </c>
-      <c r="H15" s="1"/>
+      <c r="F15">
+        <v>15</v>
+      </c>
+      <c r="G15" t="s">
+        <v>671</v>
+      </c>
+      <c r="H15" t="s">
+        <v>15</v>
+      </c>
+      <c r="J15" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
@@ -2945,9 +3074,20 @@
       <c r="E16" s="5">
         <v>101.8325</v>
       </c>
-      <c r="H16" s="1"/>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F16">
+        <v>15</v>
+      </c>
+      <c r="G16" t="s">
+        <v>671</v>
+      </c>
+      <c r="H16" t="s">
+        <v>16</v>
+      </c>
+      <c r="J16" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
         <v>32</v>
       </c>
@@ -2963,9 +3103,20 @@
       <c r="E17" s="5">
         <v>101.8325</v>
       </c>
-      <c r="H17" s="1"/>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F17">
+        <v>15</v>
+      </c>
+      <c r="G17" t="s">
+        <v>671</v>
+      </c>
+      <c r="H17" t="s">
+        <v>11</v>
+      </c>
+      <c r="J17" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A18" s="3" t="s">
         <v>33</v>
       </c>
@@ -2981,9 +3132,20 @@
       <c r="E18" s="5">
         <v>101.8325</v>
       </c>
-      <c r="H18" s="1"/>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F18">
+        <v>15</v>
+      </c>
+      <c r="G18" t="s">
+        <v>672</v>
+      </c>
+      <c r="H18" t="s">
+        <v>13</v>
+      </c>
+      <c r="J18" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="s">
         <v>34</v>
       </c>
@@ -2999,9 +3161,20 @@
       <c r="E19" s="5">
         <v>101.8325</v>
       </c>
-      <c r="H19" s="1"/>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F19">
+        <v>15</v>
+      </c>
+      <c r="G19" t="s">
+        <v>672</v>
+      </c>
+      <c r="H19" t="s">
+        <v>14</v>
+      </c>
+      <c r="J19" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A20" s="3" t="s">
         <v>35</v>
       </c>
@@ -3017,9 +3190,20 @@
       <c r="E20" s="5">
         <v>101.8325</v>
       </c>
-      <c r="H20" s="1"/>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F20">
+        <v>0</v>
+      </c>
+      <c r="G20" t="s">
+        <v>672</v>
+      </c>
+      <c r="H20" t="s">
+        <v>15</v>
+      </c>
+      <c r="J20" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A21" s="3" t="s">
         <v>36</v>
       </c>
@@ -3035,9 +3219,20 @@
       <c r="E21" s="5">
         <v>39.674999999999997</v>
       </c>
-      <c r="H21" s="1"/>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F21">
+        <v>10</v>
+      </c>
+      <c r="G21" t="s">
+        <v>672</v>
+      </c>
+      <c r="H21" t="s">
+        <v>16</v>
+      </c>
+      <c r="J21" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A22" s="3" t="s">
         <v>37</v>
       </c>
@@ -3053,9 +3248,20 @@
       <c r="E22" s="5">
         <v>417.63161374999999</v>
       </c>
-      <c r="H22" s="1"/>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F22">
+        <v>8</v>
+      </c>
+      <c r="G22" t="s">
+        <v>672</v>
+      </c>
+      <c r="H22" t="s">
+        <v>11</v>
+      </c>
+      <c r="J22" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A23" s="3" t="s">
         <v>38</v>
       </c>
@@ -3071,9 +3277,20 @@
       <c r="E23" s="5">
         <v>481.43641974999997</v>
       </c>
-      <c r="H23" s="1"/>
-    </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F23">
+        <v>5</v>
+      </c>
+      <c r="G23" t="s">
+        <v>672</v>
+      </c>
+      <c r="H23" t="s">
+        <v>13</v>
+      </c>
+      <c r="J23" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A24" s="3" t="s">
         <v>39</v>
       </c>
@@ -3089,8 +3306,20 @@
       <c r="E24" s="5">
         <v>276.40249999999997</v>
       </c>
-    </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F24">
+        <v>15</v>
+      </c>
+      <c r="G24" t="s">
+        <v>672</v>
+      </c>
+      <c r="H24" t="s">
+        <v>14</v>
+      </c>
+      <c r="J24" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A25" s="3" t="s">
         <v>40</v>
       </c>
@@ -3106,8 +3335,20 @@
       <c r="E25" s="5">
         <v>116.0097</v>
       </c>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F25">
+        <v>15</v>
+      </c>
+      <c r="G25" t="s">
+        <v>672</v>
+      </c>
+      <c r="H25" t="s">
+        <v>15</v>
+      </c>
+      <c r="J25" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A26" s="3" t="s">
         <v>41</v>
       </c>
@@ -3123,8 +3364,20 @@
       <c r="E26" s="5">
         <v>75.405643749999996</v>
       </c>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F26">
+        <v>15</v>
+      </c>
+      <c r="G26" t="s">
+        <v>672</v>
+      </c>
+      <c r="H26" t="s">
+        <v>16</v>
+      </c>
+      <c r="J26" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A27" s="3" t="s">
         <v>42</v>
       </c>
@@ -3140,8 +3393,20 @@
       <c r="E27" s="5">
         <v>101.8325</v>
       </c>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F27">
+        <v>15</v>
+      </c>
+      <c r="G27" t="s">
+        <v>672</v>
+      </c>
+      <c r="H27" t="s">
+        <v>15</v>
+      </c>
+      <c r="J27" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A28" s="3" t="s">
         <v>43</v>
       </c>
@@ -3157,8 +3422,20 @@
       <c r="E28" s="5">
         <v>251.27500000000001</v>
       </c>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F28">
+        <v>15</v>
+      </c>
+      <c r="G28" t="s">
+        <v>672</v>
+      </c>
+      <c r="H28" t="s">
+        <v>16</v>
+      </c>
+      <c r="J28" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A29" s="3" t="s">
         <v>44</v>
       </c>
@@ -3174,8 +3451,20 @@
       <c r="E29" s="5">
         <v>296.24</v>
       </c>
-    </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F29">
+        <v>15</v>
+      </c>
+      <c r="G29" t="s">
+        <v>673</v>
+      </c>
+      <c r="H29" t="s">
+        <v>11</v>
+      </c>
+      <c r="J29" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A30" s="3" t="s">
         <v>45</v>
       </c>
@@ -3191,8 +3480,20 @@
       <c r="E30" s="5">
         <v>1653.125</v>
       </c>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F30">
+        <v>15</v>
+      </c>
+      <c r="G30" t="s">
+        <v>673</v>
+      </c>
+      <c r="H30" t="s">
+        <v>13</v>
+      </c>
+      <c r="J30" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A31" s="3" t="s">
         <v>46</v>
       </c>
@@ -3208,8 +3509,20 @@
       <c r="E31" s="5">
         <v>395.75812500000001</v>
       </c>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F31">
+        <v>15</v>
+      </c>
+      <c r="G31" t="s">
+        <v>673</v>
+      </c>
+      <c r="H31" t="s">
+        <v>14</v>
+      </c>
+      <c r="J31" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A32" s="3" t="s">
         <v>47</v>
       </c>
@@ -3225,8 +3538,20 @@
       <c r="E32" s="5">
         <v>207.301875</v>
       </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F32">
+        <v>15</v>
+      </c>
+      <c r="G32" t="s">
+        <v>673</v>
+      </c>
+      <c r="H32" t="s">
+        <v>15</v>
+      </c>
+      <c r="J32" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A33" s="3" t="s">
         <v>48</v>
       </c>
@@ -3242,8 +3567,20 @@
       <c r="E33" s="5">
         <v>121.80925925</v>
       </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F33">
+        <v>15</v>
+      </c>
+      <c r="G33" t="s">
+        <v>673</v>
+      </c>
+      <c r="H33" t="s">
+        <v>16</v>
+      </c>
+      <c r="J33" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A34" s="3" t="s">
         <v>49</v>
       </c>
@@ -3259,8 +3596,20 @@
       <c r="E34" s="5">
         <v>110.29650000000001</v>
       </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F34">
+        <v>15</v>
+      </c>
+      <c r="G34" t="s">
+        <v>673</v>
+      </c>
+      <c r="H34" t="s">
+        <v>11</v>
+      </c>
+      <c r="J34" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A35" s="3" t="s">
         <v>50</v>
       </c>
@@ -3276,8 +3625,20 @@
       <c r="E35" s="5">
         <v>232.00617500000001</v>
       </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F35">
+        <v>0</v>
+      </c>
+      <c r="G35" t="s">
+        <v>673</v>
+      </c>
+      <c r="H35" t="s">
+        <v>13</v>
+      </c>
+      <c r="J35" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A36" s="3" t="s">
         <v>51</v>
       </c>
@@ -3293,8 +3654,20 @@
       <c r="E36" s="5">
         <v>382.82896825000006</v>
       </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F36">
+        <v>10</v>
+      </c>
+      <c r="G36" t="s">
+        <v>673</v>
+      </c>
+      <c r="H36" t="s">
+        <v>14</v>
+      </c>
+      <c r="J36" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A37" s="3" t="s">
         <v>52</v>
       </c>
@@ -3310,8 +3683,20 @@
       <c r="E37" s="5">
         <v>276.40249999999997</v>
       </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F37">
+        <v>8</v>
+      </c>
+      <c r="G37" t="s">
+        <v>673</v>
+      </c>
+      <c r="H37" t="s">
+        <v>15</v>
+      </c>
+      <c r="J37" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A38" s="3" t="s">
         <v>53</v>
       </c>
@@ -3327,8 +3712,20 @@
       <c r="E38" s="5">
         <v>238.71124999999998</v>
       </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F38">
+        <v>5</v>
+      </c>
+      <c r="G38" t="s">
+        <v>674</v>
+      </c>
+      <c r="H38" t="s">
+        <v>16</v>
+      </c>
+      <c r="J38" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A39" s="3" t="s">
         <v>54</v>
       </c>
@@ -3344,8 +3741,20 @@
       <c r="E39" s="5">
         <v>185.15</v>
       </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F39">
+        <v>15</v>
+      </c>
+      <c r="G39" t="s">
+        <v>674</v>
+      </c>
+      <c r="H39" t="s">
+        <v>11</v>
+      </c>
+      <c r="J39" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A40" s="3" t="s">
         <v>55</v>
       </c>
@@ -3361,8 +3770,20 @@
       <c r="E40" s="5">
         <v>188.45625000000001</v>
       </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F40">
+        <v>15</v>
+      </c>
+      <c r="G40" t="s">
+        <v>674</v>
+      </c>
+      <c r="H40" t="s">
+        <v>13</v>
+      </c>
+      <c r="J40" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A41" s="3" t="s">
         <v>56</v>
       </c>
@@ -3378,8 +3799,20 @@
       <c r="E41" s="5">
         <v>188.45625000000001</v>
       </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F41">
+        <v>15</v>
+      </c>
+      <c r="G41" t="s">
+        <v>674</v>
+      </c>
+      <c r="H41" t="s">
+        <v>14</v>
+      </c>
+      <c r="J41" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A42" s="3" t="s">
         <v>57</v>
       </c>
@@ -3395,8 +3828,20 @@
       <c r="E42" s="5">
         <v>188.45625000000001</v>
       </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F42">
+        <v>15</v>
+      </c>
+      <c r="G42" t="s">
+        <v>674</v>
+      </c>
+      <c r="H42" t="s">
+        <v>15</v>
+      </c>
+      <c r="J42" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A43" s="3" t="s">
         <v>58</v>
       </c>
@@ -3412,8 +3857,20 @@
       <c r="E43" s="5">
         <v>188.45625000000001</v>
       </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F43">
+        <v>15</v>
+      </c>
+      <c r="G43" t="s">
+        <v>674</v>
+      </c>
+      <c r="H43" t="s">
+        <v>16</v>
+      </c>
+      <c r="J43" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A44" s="3" t="s">
         <v>59</v>
       </c>
@@ -3429,8 +3886,20 @@
       <c r="E44" s="5">
         <v>188.45625000000001</v>
       </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F44">
+        <v>15</v>
+      </c>
+      <c r="G44" t="s">
+        <v>674</v>
+      </c>
+      <c r="H44" t="s">
+        <v>11</v>
+      </c>
+      <c r="J44" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A45" s="3" t="s">
         <v>60</v>
       </c>
@@ -3446,8 +3915,20 @@
       <c r="E45" s="5">
         <v>188.45625000000001</v>
       </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F45">
+        <v>15</v>
+      </c>
+      <c r="G45" t="s">
+        <v>674</v>
+      </c>
+      <c r="H45" t="s">
+        <v>13</v>
+      </c>
+      <c r="J45" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A46" s="3" t="s">
         <v>61</v>
       </c>
@@ -3463,8 +3944,20 @@
       <c r="E46" s="5">
         <v>396.75</v>
       </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F46">
+        <v>0</v>
+      </c>
+      <c r="G46" t="s">
+        <v>674</v>
+      </c>
+      <c r="H46" t="s">
+        <v>14</v>
+      </c>
+      <c r="J46" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A47" s="3" t="s">
         <v>62</v>
       </c>
@@ -3480,8 +3973,20 @@
       <c r="E47" s="5">
         <v>244.66249999999999</v>
       </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F47">
+        <v>10</v>
+      </c>
+      <c r="G47" t="s">
+        <v>675</v>
+      </c>
+      <c r="H47" t="s">
+        <v>15</v>
+      </c>
+      <c r="J47" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A48" s="3" t="s">
         <v>63</v>
       </c>
@@ -3497,8 +4002,20 @@
       <c r="E48" s="5">
         <v>244.66249999999999</v>
       </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F48">
+        <v>8</v>
+      </c>
+      <c r="G48" t="s">
+        <v>675</v>
+      </c>
+      <c r="H48" t="s">
+        <v>16</v>
+      </c>
+      <c r="J48" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A49" s="3" t="s">
         <v>64</v>
       </c>
@@ -3514,8 +4031,20 @@
       <c r="E49" s="5">
         <v>238.05</v>
       </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F49">
+        <v>5</v>
+      </c>
+      <c r="G49" t="s">
+        <v>675</v>
+      </c>
+      <c r="H49" t="s">
+        <v>16</v>
+      </c>
+      <c r="J49" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A50" s="3" t="s">
         <v>65</v>
       </c>
@@ -3531,8 +4060,20 @@
       <c r="E50" s="5">
         <v>158.69999999999999</v>
       </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F50">
+        <v>15</v>
+      </c>
+      <c r="G50" t="s">
+        <v>675</v>
+      </c>
+      <c r="H50" t="s">
+        <v>11</v>
+      </c>
+      <c r="J50" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A51" s="3" t="s">
         <v>66</v>
       </c>
@@ -3548,8 +4089,20 @@
       <c r="E51" s="5">
         <v>152.08750000000001</v>
       </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F51">
+        <v>15</v>
+      </c>
+      <c r="G51" t="s">
+        <v>675</v>
+      </c>
+      <c r="H51" t="s">
+        <v>13</v>
+      </c>
+      <c r="J51" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A52" s="3" t="s">
         <v>67</v>
       </c>
@@ -3565,8 +4118,20 @@
       <c r="E52" s="5">
         <v>112.41249999999999</v>
       </c>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F52">
+        <v>15</v>
+      </c>
+      <c r="G52" t="s">
+        <v>675</v>
+      </c>
+      <c r="H52" t="s">
+        <v>14</v>
+      </c>
+      <c r="J52" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A53" s="3" t="s">
         <v>68</v>
       </c>
@@ -3582,8 +4147,20 @@
       <c r="E53" s="5">
         <v>218.21250000000001</v>
       </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F53">
+        <v>15</v>
+      </c>
+      <c r="G53" t="s">
+        <v>675</v>
+      </c>
+      <c r="H53" t="s">
+        <v>15</v>
+      </c>
+      <c r="J53" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A54" s="3" t="s">
         <v>69</v>
       </c>
@@ -3599,8 +4176,20 @@
       <c r="E54" s="5">
         <v>92.575000000000003</v>
       </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F54">
+        <v>15</v>
+      </c>
+      <c r="G54" t="s">
+        <v>675</v>
+      </c>
+      <c r="H54" t="s">
+        <v>16</v>
+      </c>
+      <c r="J54" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A55" s="3" t="s">
         <v>70</v>
       </c>
@@ -3616,8 +4205,20 @@
       <c r="E55" s="5">
         <v>59.512500000000003</v>
       </c>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F55">
+        <v>15</v>
+      </c>
+      <c r="G55" t="s">
+        <v>671</v>
+      </c>
+      <c r="H55" t="s">
+        <v>16</v>
+      </c>
+      <c r="J55" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A56" s="3" t="s">
         <v>71</v>
       </c>
@@ -3633,8 +4234,20 @@
       <c r="E56" s="5">
         <v>145.47499999999999</v>
       </c>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F56">
+        <v>0</v>
+      </c>
+      <c r="G56" t="s">
+        <v>671</v>
+      </c>
+      <c r="H56" t="s">
+        <v>11</v>
+      </c>
+      <c r="J56" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A57" s="3" t="s">
         <v>72</v>
       </c>
@@ -3650,8 +4263,20 @@
       <c r="E57" s="5">
         <v>317.39999999999998</v>
       </c>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F57">
+        <v>10</v>
+      </c>
+      <c r="G57" t="s">
+        <v>671</v>
+      </c>
+      <c r="H57" t="s">
+        <v>13</v>
+      </c>
+      <c r="J57" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A58" s="3" t="s">
         <v>73</v>
       </c>
@@ -3667,8 +4292,20 @@
       <c r="E58" s="5">
         <v>482.71249999999998</v>
       </c>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F58">
+        <v>8</v>
+      </c>
+      <c r="G58" t="s">
+        <v>671</v>
+      </c>
+      <c r="H58" t="s">
+        <v>14</v>
+      </c>
+      <c r="J58" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A59" s="3" t="s">
         <v>74</v>
       </c>
@@ -3684,8 +4321,20 @@
       <c r="E59" s="5">
         <v>462.875</v>
       </c>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F59">
+        <v>5</v>
+      </c>
+      <c r="G59" t="s">
+        <v>671</v>
+      </c>
+      <c r="H59" t="s">
+        <v>15</v>
+      </c>
+      <c r="J59" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A60" s="3" t="s">
         <v>75</v>
       </c>
@@ -3701,8 +4350,20 @@
       <c r="E60" s="5">
         <v>296.24</v>
       </c>
-    </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F60">
+        <v>15</v>
+      </c>
+      <c r="G60" t="s">
+        <v>671</v>
+      </c>
+      <c r="H60" t="s">
+        <v>16</v>
+      </c>
+      <c r="J60" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A61" s="3" t="s">
         <v>76</v>
       </c>
@@ -3718,8 +4379,23 @@
       <c r="E61" s="5">
         <v>357.07499999999999</v>
       </c>
-    </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F61">
+        <v>15</v>
+      </c>
+      <c r="G61" t="s">
+        <v>12</v>
+      </c>
+      <c r="H61" t="s">
+        <v>11</v>
+      </c>
+      <c r="I61" t="s">
+        <v>10</v>
+      </c>
+      <c r="J61" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A62" s="3" t="s">
         <v>77</v>
       </c>
@@ -3735,8 +4411,20 @@
       <c r="E62" s="5">
         <v>239.3725</v>
       </c>
-    </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F62">
+        <v>15</v>
+      </c>
+      <c r="G62" t="s">
+        <v>12</v>
+      </c>
+      <c r="H62" t="s">
+        <v>13</v>
+      </c>
+      <c r="J62" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="63" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A63" s="3" t="s">
         <v>78</v>
       </c>
@@ -3752,8 +4440,20 @@
       <c r="E63" s="5">
         <v>239.3725</v>
       </c>
-    </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F63">
+        <v>15</v>
+      </c>
+      <c r="G63" t="s">
+        <v>12</v>
+      </c>
+      <c r="H63" t="s">
+        <v>14</v>
+      </c>
+      <c r="J63" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A64" s="3" t="s">
         <v>79</v>
       </c>
@@ -3769,8 +4469,20 @@
       <c r="E64" s="5">
         <v>230.11499999999998</v>
       </c>
-    </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F64">
+        <v>15</v>
+      </c>
+      <c r="G64" t="s">
+        <v>12</v>
+      </c>
+      <c r="H64" t="s">
+        <v>15</v>
+      </c>
+      <c r="J64" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="65" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A65" s="3" t="s">
         <v>80</v>
       </c>
@@ -3786,8 +4498,20 @@
       <c r="E65" s="5">
         <v>462.875</v>
       </c>
-    </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F65">
+        <v>15</v>
+      </c>
+      <c r="G65" t="s">
+        <v>12</v>
+      </c>
+      <c r="H65" t="s">
+        <v>16</v>
+      </c>
+      <c r="J65" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="66" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A66" s="3" t="s">
         <v>81</v>
       </c>
@@ -3803,8 +4527,20 @@
       <c r="E66" s="5">
         <v>370.3</v>
       </c>
-    </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F66">
+        <v>15</v>
+      </c>
+      <c r="G66" t="s">
+        <v>671</v>
+      </c>
+      <c r="H66" t="s">
+        <v>11</v>
+      </c>
+      <c r="J66" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="67" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A67" s="3" t="s">
         <v>82</v>
       </c>
@@ -3820,8 +4556,20 @@
       <c r="E67" s="5">
         <v>148.78125</v>
       </c>
-    </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F67">
+        <v>15</v>
+      </c>
+      <c r="G67" t="s">
+        <v>671</v>
+      </c>
+      <c r="H67" t="s">
+        <v>13</v>
+      </c>
+      <c r="J67" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="68" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A68" s="3" t="s">
         <v>83</v>
       </c>
@@ -3837,8 +4585,20 @@
       <c r="E68" s="5">
         <v>168.61875000000001</v>
       </c>
-    </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F68">
+        <v>15</v>
+      </c>
+      <c r="G68" t="s">
+        <v>671</v>
+      </c>
+      <c r="H68" t="s">
+        <v>14</v>
+      </c>
+      <c r="J68" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="69" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A69" s="3" t="s">
         <v>84</v>
       </c>
@@ -3854,8 +4614,20 @@
       <c r="E69" s="5">
         <v>168.61875000000001</v>
       </c>
-    </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F69">
+        <v>15</v>
+      </c>
+      <c r="G69" t="s">
+        <v>671</v>
+      </c>
+      <c r="H69" t="s">
+        <v>15</v>
+      </c>
+      <c r="J69" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="70" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A70" s="3" t="s">
         <v>85</v>
       </c>
@@ -3871,8 +4643,20 @@
       <c r="E70" s="5">
         <v>376.91250000000002</v>
       </c>
-    </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F70">
+        <v>15</v>
+      </c>
+      <c r="G70" t="s">
+        <v>671</v>
+      </c>
+      <c r="H70" t="s">
+        <v>16</v>
+      </c>
+      <c r="J70" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="71" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A71" s="3" t="s">
         <v>86</v>
       </c>
@@ -3888,8 +4672,20 @@
       <c r="E71" s="5">
         <v>469.48750000000001</v>
       </c>
-    </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F71">
+        <v>15</v>
+      </c>
+      <c r="G71" t="s">
+        <v>671</v>
+      </c>
+      <c r="H71" t="s">
+        <v>11</v>
+      </c>
+      <c r="J71" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="72" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A72" s="3" t="s">
         <v>87</v>
       </c>
@@ -3905,8 +4701,20 @@
       <c r="E72" s="5">
         <v>277.72500000000002</v>
       </c>
-    </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F72">
+        <v>15</v>
+      </c>
+      <c r="G72" t="s">
+        <v>671</v>
+      </c>
+      <c r="H72" t="s">
+        <v>13</v>
+      </c>
+      <c r="J72" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="73" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A73" s="3" t="s">
         <v>88</v>
       </c>
@@ -3922,8 +4730,20 @@
       <c r="E73" s="5">
         <v>816.64374999999995</v>
       </c>
-    </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F73">
+        <v>15</v>
+      </c>
+      <c r="G73" t="s">
+        <v>671</v>
+      </c>
+      <c r="H73" t="s">
+        <v>14</v>
+      </c>
+      <c r="J73" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="74" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A74" s="3" t="s">
         <v>89</v>
       </c>
@@ -3939,8 +4759,20 @@
       <c r="E74" s="5">
         <v>92.575000000000003</v>
       </c>
-    </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F74">
+        <v>0</v>
+      </c>
+      <c r="G74" t="s">
+        <v>671</v>
+      </c>
+      <c r="H74" t="s">
+        <v>15</v>
+      </c>
+      <c r="J74" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="75" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A75" s="3" t="s">
         <v>90</v>
       </c>
@@ -3956,8 +4788,20 @@
       <c r="E75" s="5">
         <v>42.319999999999993</v>
       </c>
-    </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F75">
+        <v>10</v>
+      </c>
+      <c r="G75" t="s">
+        <v>671</v>
+      </c>
+      <c r="H75" t="s">
+        <v>16</v>
+      </c>
+      <c r="J75" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="76" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A76" s="3" t="s">
         <v>91</v>
       </c>
@@ -3973,8 +4817,20 @@
       <c r="E76" s="5">
         <v>128.2825</v>
       </c>
-    </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F76">
+        <v>8</v>
+      </c>
+      <c r="G76" t="s">
+        <v>671</v>
+      </c>
+      <c r="H76" t="s">
+        <v>11</v>
+      </c>
+      <c r="J76" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="77" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A77" s="3" t="s">
         <v>92</v>
       </c>
@@ -3990,8 +4846,20 @@
       <c r="E77" s="5">
         <v>249.95249999999999</v>
       </c>
-    </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F77">
+        <v>5</v>
+      </c>
+      <c r="G77" t="s">
+        <v>672</v>
+      </c>
+      <c r="H77" t="s">
+        <v>13</v>
+      </c>
+      <c r="J77" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="78" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A78" s="3" t="s">
         <v>93</v>
       </c>
@@ -4007,8 +4875,20 @@
       <c r="E78" s="5">
         <v>129.60500000000002</v>
       </c>
-    </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F78">
+        <v>15</v>
+      </c>
+      <c r="G78" t="s">
+        <v>672</v>
+      </c>
+      <c r="H78" t="s">
+        <v>14</v>
+      </c>
+      <c r="J78" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="79" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A79" s="3" t="s">
         <v>94</v>
       </c>
@@ -4024,8 +4904,20 @@
       <c r="E79" s="5">
         <v>112.41249999999999</v>
       </c>
-    </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F79">
+        <v>15</v>
+      </c>
+      <c r="G79" t="s">
+        <v>672</v>
+      </c>
+      <c r="H79" t="s">
+        <v>15</v>
+      </c>
+      <c r="J79" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="80" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A80" s="3" t="s">
         <v>95</v>
       </c>
@@ -4041,8 +4933,20 @@
       <c r="E80" s="5">
         <v>409.97500000000002</v>
       </c>
-    </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F80">
+        <v>15</v>
+      </c>
+      <c r="G80" t="s">
+        <v>672</v>
+      </c>
+      <c r="H80" t="s">
+        <v>16</v>
+      </c>
+      <c r="J80" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="81" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A81" s="3" t="s">
         <v>96</v>
       </c>
@@ -4058,8 +4962,20 @@
       <c r="E81" s="5">
         <v>767.05</v>
       </c>
-    </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F81">
+        <v>15</v>
+      </c>
+      <c r="G81" t="s">
+        <v>672</v>
+      </c>
+      <c r="H81" t="s">
+        <v>11</v>
+      </c>
+      <c r="J81" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="82" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A82" s="3" t="s">
         <v>97</v>
       </c>
@@ -4075,8 +4991,20 @@
       <c r="E82" s="5">
         <v>767.05</v>
       </c>
-    </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F82">
+        <v>15</v>
+      </c>
+      <c r="G82" t="s">
+        <v>672</v>
+      </c>
+      <c r="H82" t="s">
+        <v>13</v>
+      </c>
+      <c r="J82" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="83" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A83" s="3" t="s">
         <v>98</v>
       </c>
@@ -4092,8 +5020,20 @@
       <c r="E83" s="5">
         <v>74.06</v>
       </c>
-    </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F83">
+        <v>15</v>
+      </c>
+      <c r="G83" t="s">
+        <v>672</v>
+      </c>
+      <c r="H83" t="s">
+        <v>14</v>
+      </c>
+      <c r="J83" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="84" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A84" s="3" t="s">
         <v>99</v>
       </c>
@@ -4109,8 +5049,20 @@
       <c r="E84" s="5">
         <v>66.125</v>
       </c>
-    </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F84">
+        <v>15</v>
+      </c>
+      <c r="G84" t="s">
+        <v>672</v>
+      </c>
+      <c r="H84" t="s">
+        <v>15</v>
+      </c>
+      <c r="J84" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="85" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A85" s="3" t="s">
         <v>100</v>
       </c>
@@ -4126,8 +5078,20 @@
       <c r="E85" s="5">
         <v>296.24</v>
       </c>
-    </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F85">
+        <v>15</v>
+      </c>
+      <c r="G85" t="s">
+        <v>672</v>
+      </c>
+      <c r="H85" t="s">
+        <v>16</v>
+      </c>
+      <c r="J85" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="86" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A86" s="3" t="s">
         <v>101</v>
       </c>
@@ -4143,8 +5107,20 @@
       <c r="E86" s="5">
         <v>462.875</v>
       </c>
-    </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F86">
+        <v>15</v>
+      </c>
+      <c r="G86" t="s">
+        <v>672</v>
+      </c>
+      <c r="H86" t="s">
+        <v>15</v>
+      </c>
+      <c r="J86" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="87" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A87" s="3" t="s">
         <v>102</v>
       </c>
@@ -4160,8 +5136,20 @@
       <c r="E87" s="5">
         <v>376.91250000000002</v>
       </c>
-    </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F87">
+        <v>15</v>
+      </c>
+      <c r="G87" t="s">
+        <v>672</v>
+      </c>
+      <c r="H87" t="s">
+        <v>16</v>
+      </c>
+      <c r="J87" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="88" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A88" s="3" t="s">
         <v>103</v>
       </c>
@@ -4177,8 +5165,20 @@
       <c r="E88" s="5">
         <v>101.8325</v>
       </c>
-    </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F88">
+        <v>15</v>
+      </c>
+      <c r="G88" t="s">
+        <v>673</v>
+      </c>
+      <c r="H88" t="s">
+        <v>11</v>
+      </c>
+      <c r="J88" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="89" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A89" s="3" t="s">
         <v>104</v>
       </c>
@@ -4194,8 +5194,20 @@
       <c r="E89" s="5">
         <v>101.8325</v>
       </c>
-    </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F89">
+        <v>15</v>
+      </c>
+      <c r="G89" t="s">
+        <v>673</v>
+      </c>
+      <c r="H89" t="s">
+        <v>13</v>
+      </c>
+      <c r="J89" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="90" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A90" s="3" t="s">
         <v>105</v>
       </c>
@@ -4211,8 +5223,20 @@
       <c r="E90" s="5">
         <v>101.8325</v>
       </c>
-    </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F90">
+        <v>15</v>
+      </c>
+      <c r="G90" t="s">
+        <v>673</v>
+      </c>
+      <c r="H90" t="s">
+        <v>14</v>
+      </c>
+      <c r="J90" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="91" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A91" s="3" t="s">
         <v>106</v>
       </c>
@@ -4228,8 +5252,20 @@
       <c r="E91" s="5">
         <v>101.8325</v>
       </c>
-    </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F91">
+        <v>0</v>
+      </c>
+      <c r="G91" t="s">
+        <v>673</v>
+      </c>
+      <c r="H91" t="s">
+        <v>15</v>
+      </c>
+      <c r="J91" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="92" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A92" s="3" t="s">
         <v>107</v>
       </c>
@@ -4245,8 +5281,20 @@
       <c r="E92" s="5">
         <v>133.30799999999999</v>
       </c>
-    </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F92">
+        <v>10</v>
+      </c>
+      <c r="G92" t="s">
+        <v>673</v>
+      </c>
+      <c r="H92" t="s">
+        <v>16</v>
+      </c>
+      <c r="J92" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="93" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A93" s="3" t="s">
         <v>108</v>
       </c>
@@ -4262,8 +5310,20 @@
       <c r="E93" s="5">
         <v>133.30799999999999</v>
       </c>
-    </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F93">
+        <v>8</v>
+      </c>
+      <c r="G93" t="s">
+        <v>673</v>
+      </c>
+      <c r="H93" t="s">
+        <v>11</v>
+      </c>
+      <c r="J93" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="94" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A94" s="3" t="s">
         <v>109</v>
       </c>
@@ -4279,8 +5339,20 @@
       <c r="E94" s="5">
         <v>133.30799999999999</v>
       </c>
-    </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F94">
+        <v>5</v>
+      </c>
+      <c r="G94" t="s">
+        <v>673</v>
+      </c>
+      <c r="H94" t="s">
+        <v>13</v>
+      </c>
+      <c r="J94" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="95" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A95" s="3" t="s">
         <v>110</v>
       </c>
@@ -4296,8 +5368,20 @@
       <c r="E95" s="5">
         <v>133.30799999999999</v>
       </c>
-    </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F95">
+        <v>15</v>
+      </c>
+      <c r="G95" t="s">
+        <v>673</v>
+      </c>
+      <c r="H95" t="s">
+        <v>14</v>
+      </c>
+      <c r="J95" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="96" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A96" s="3" t="s">
         <v>111</v>
       </c>
@@ -4313,8 +5397,20 @@
       <c r="E96" s="5">
         <v>133.30799999999999</v>
       </c>
-    </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F96">
+        <v>15</v>
+      </c>
+      <c r="G96" t="s">
+        <v>673</v>
+      </c>
+      <c r="H96" t="s">
+        <v>15</v>
+      </c>
+      <c r="J96" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="97" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A97" s="3" t="s">
         <v>112</v>
       </c>
@@ -4330,8 +5426,20 @@
       <c r="E97" s="5">
         <v>133.30799999999999</v>
       </c>
-    </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F97">
+        <v>15</v>
+      </c>
+      <c r="G97" t="s">
+        <v>674</v>
+      </c>
+      <c r="H97" t="s">
+        <v>16</v>
+      </c>
+      <c r="J97" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="98" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A98" s="3" t="s">
         <v>113</v>
       </c>
@@ -4347,8 +5455,20 @@
       <c r="E98" s="5">
         <v>133.30799999999999</v>
       </c>
-    </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F98">
+        <v>15</v>
+      </c>
+      <c r="G98" t="s">
+        <v>674</v>
+      </c>
+      <c r="H98" t="s">
+        <v>11</v>
+      </c>
+      <c r="J98" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="99" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A99" s="3" t="s">
         <v>114</v>
       </c>
@@ -4364,8 +5484,20 @@
       <c r="E99" s="5">
         <v>76.176000000000016</v>
       </c>
-    </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F99">
+        <v>15</v>
+      </c>
+      <c r="G99" t="s">
+        <v>674</v>
+      </c>
+      <c r="H99" t="s">
+        <v>13</v>
+      </c>
+      <c r="J99" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="100" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A100" s="3" t="s">
         <v>115</v>
       </c>
@@ -4381,8 +5513,20 @@
       <c r="E100" s="5">
         <v>76.176000000000016</v>
       </c>
-    </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F100">
+        <v>15</v>
+      </c>
+      <c r="G100" t="s">
+        <v>674</v>
+      </c>
+      <c r="H100" t="s">
+        <v>14</v>
+      </c>
+      <c r="J100" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="101" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A101" s="3" t="s">
         <v>116</v>
       </c>
@@ -4398,8 +5542,20 @@
       <c r="E101" s="5">
         <v>76.176000000000016</v>
       </c>
-    </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F101">
+        <v>15</v>
+      </c>
+      <c r="G101" t="s">
+        <v>674</v>
+      </c>
+      <c r="H101" t="s">
+        <v>15</v>
+      </c>
+      <c r="J101" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="102" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A102" s="3" t="s">
         <v>117</v>
       </c>
@@ -4415,8 +5571,20 @@
       <c r="E102" s="5">
         <v>76.176000000000016</v>
       </c>
-    </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F102">
+        <v>15</v>
+      </c>
+      <c r="G102" t="s">
+        <v>674</v>
+      </c>
+      <c r="H102" t="s">
+        <v>16</v>
+      </c>
+      <c r="J102" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="103" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A103" s="3" t="s">
         <v>118</v>
       </c>
@@ -4432,8 +5600,20 @@
       <c r="E103" s="5">
         <v>76.176000000000016</v>
       </c>
-    </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F103">
+        <v>15</v>
+      </c>
+      <c r="G103" t="s">
+        <v>674</v>
+      </c>
+      <c r="H103" t="s">
+        <v>11</v>
+      </c>
+      <c r="J103" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="104" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A104" s="3" t="s">
         <v>119</v>
       </c>
@@ -4449,8 +5629,20 @@
       <c r="E104" s="5">
         <v>76.176000000000016</v>
       </c>
-    </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F104">
+        <v>15</v>
+      </c>
+      <c r="G104" t="s">
+        <v>674</v>
+      </c>
+      <c r="H104" t="s">
+        <v>13</v>
+      </c>
+      <c r="J104" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="105" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A105" s="3" t="s">
         <v>120</v>
       </c>
@@ -4466,8 +5658,20 @@
       <c r="E105" s="5">
         <v>76.176000000000016</v>
       </c>
-    </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F105">
+        <v>0</v>
+      </c>
+      <c r="G105" t="s">
+        <v>674</v>
+      </c>
+      <c r="H105" t="s">
+        <v>14</v>
+      </c>
+      <c r="J105" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="106" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A106" s="3" t="s">
         <v>121</v>
       </c>
@@ -4483,8 +5687,20 @@
       <c r="E106" s="5">
         <v>76.176000000000016</v>
       </c>
-    </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F106">
+        <v>10</v>
+      </c>
+      <c r="G106" t="s">
+        <v>675</v>
+      </c>
+      <c r="H106" t="s">
+        <v>15</v>
+      </c>
+      <c r="J106" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="107" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A107" s="3" t="s">
         <v>122</v>
       </c>
@@ -4500,8 +5716,20 @@
       <c r="E107" s="5">
         <v>76.176000000000016</v>
       </c>
-    </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F107">
+        <v>8</v>
+      </c>
+      <c r="G107" t="s">
+        <v>675</v>
+      </c>
+      <c r="H107" t="s">
+        <v>16</v>
+      </c>
+      <c r="J107" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="108" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A108" s="3" t="s">
         <v>123</v>
       </c>
@@ -4517,8 +5745,20 @@
       <c r="E108" s="5">
         <v>76.176000000000016</v>
       </c>
-    </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F108">
+        <v>5</v>
+      </c>
+      <c r="G108" t="s">
+        <v>675</v>
+      </c>
+      <c r="H108" t="s">
+        <v>16</v>
+      </c>
+      <c r="J108" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="109" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A109" s="3" t="s">
         <v>124</v>
       </c>
@@ -4534,8 +5774,20 @@
       <c r="E109" s="5">
         <v>76.176000000000016</v>
       </c>
-    </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F109">
+        <v>15</v>
+      </c>
+      <c r="G109" t="s">
+        <v>675</v>
+      </c>
+      <c r="H109" t="s">
+        <v>11</v>
+      </c>
+      <c r="J109" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="110" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A110" s="3" t="s">
         <v>125</v>
       </c>
@@ -4551,8 +5803,20 @@
       <c r="E110" s="5">
         <v>76.176000000000016</v>
       </c>
-    </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F110">
+        <v>15</v>
+      </c>
+      <c r="G110" t="s">
+        <v>675</v>
+      </c>
+      <c r="H110" t="s">
+        <v>13</v>
+      </c>
+      <c r="J110" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="111" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A111" s="3" t="s">
         <v>126</v>
       </c>
@@ -4568,8 +5832,20 @@
       <c r="E111" s="5">
         <v>76.176000000000016</v>
       </c>
-    </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F111">
+        <v>15</v>
+      </c>
+      <c r="G111" t="s">
+        <v>675</v>
+      </c>
+      <c r="H111" t="s">
+        <v>14</v>
+      </c>
+      <c r="J111" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="112" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A112" s="3" t="s">
         <v>127</v>
       </c>
@@ -4585,8 +5861,20 @@
       <c r="E112" s="5">
         <v>76.176000000000016</v>
       </c>
-    </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F112">
+        <v>15</v>
+      </c>
+      <c r="G112" t="s">
+        <v>675</v>
+      </c>
+      <c r="H112" t="s">
+        <v>15</v>
+      </c>
+      <c r="J112" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="113" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A113" s="3" t="s">
         <v>128</v>
       </c>
@@ -4602,8 +5890,20 @@
       <c r="E113" s="5">
         <v>76.176000000000016</v>
       </c>
-    </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F113">
+        <v>15</v>
+      </c>
+      <c r="G113" t="s">
+        <v>675</v>
+      </c>
+      <c r="H113" t="s">
+        <v>16</v>
+      </c>
+      <c r="J113" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="114" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A114" s="3" t="s">
         <v>129</v>
       </c>
@@ -4619,8 +5919,20 @@
       <c r="E114" s="5">
         <v>76.176000000000016</v>
       </c>
-    </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F114">
+        <v>15</v>
+      </c>
+      <c r="G114" t="s">
+        <v>671</v>
+      </c>
+      <c r="H114" t="s">
+        <v>16</v>
+      </c>
+      <c r="J114" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="115" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A115" s="3" t="s">
         <v>130</v>
       </c>
@@ -4636,8 +5948,20 @@
       <c r="E115" s="5">
         <v>76.176000000000016</v>
       </c>
-    </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F115">
+        <v>15</v>
+      </c>
+      <c r="G115" t="s">
+        <v>671</v>
+      </c>
+      <c r="H115" t="s">
+        <v>11</v>
+      </c>
+      <c r="J115" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="116" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A116" s="3" t="s">
         <v>131</v>
       </c>
@@ -4653,8 +5977,20 @@
       <c r="E116" s="5">
         <v>76.176000000000016</v>
       </c>
-    </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F116">
+        <v>0</v>
+      </c>
+      <c r="G116" t="s">
+        <v>671</v>
+      </c>
+      <c r="H116" t="s">
+        <v>13</v>
+      </c>
+      <c r="J116" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="117" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A117" s="3" t="s">
         <v>132</v>
       </c>
@@ -4670,8 +6006,20 @@
       <c r="E117" s="5">
         <v>76.176000000000016</v>
       </c>
-    </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F117">
+        <v>10</v>
+      </c>
+      <c r="G117" t="s">
+        <v>671</v>
+      </c>
+      <c r="H117" t="s">
+        <v>14</v>
+      </c>
+      <c r="J117" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="118" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A118" s="3" t="s">
         <v>133</v>
       </c>
@@ -4687,8 +6035,20 @@
       <c r="E118" s="5">
         <v>76.176000000000016</v>
       </c>
-    </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F118">
+        <v>8</v>
+      </c>
+      <c r="G118" t="s">
+        <v>671</v>
+      </c>
+      <c r="H118" t="s">
+        <v>15</v>
+      </c>
+      <c r="J118" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="119" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A119" s="3" t="s">
         <v>134</v>
       </c>
@@ -4704,8 +6064,20 @@
       <c r="E119" s="5">
         <v>76.176000000000016</v>
       </c>
-    </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F119">
+        <v>5</v>
+      </c>
+      <c r="G119" t="s">
+        <v>671</v>
+      </c>
+      <c r="H119" t="s">
+        <v>16</v>
+      </c>
+      <c r="J119" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="120" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A120" s="3" t="s">
         <v>135</v>
       </c>
@@ -4721,8 +6093,23 @@
       <c r="E120" s="5">
         <v>76.176000000000016</v>
       </c>
-    </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F120">
+        <v>15</v>
+      </c>
+      <c r="G120" t="s">
+        <v>12</v>
+      </c>
+      <c r="H120" t="s">
+        <v>11</v>
+      </c>
+      <c r="I120" t="s">
+        <v>10</v>
+      </c>
+      <c r="J120" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="121" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A121" s="3" t="s">
         <v>136</v>
       </c>
@@ -4738,8 +6125,20 @@
       <c r="E121" s="5">
         <v>76.176000000000016</v>
       </c>
-    </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F121">
+        <v>15</v>
+      </c>
+      <c r="G121" t="s">
+        <v>12</v>
+      </c>
+      <c r="H121" t="s">
+        <v>13</v>
+      </c>
+      <c r="J121" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="122" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A122" s="3" t="s">
         <v>137</v>
       </c>
@@ -4755,8 +6154,20 @@
       <c r="E122" s="5">
         <v>76.176000000000016</v>
       </c>
-    </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F122">
+        <v>15</v>
+      </c>
+      <c r="G122" t="s">
+        <v>12</v>
+      </c>
+      <c r="H122" t="s">
+        <v>14</v>
+      </c>
+      <c r="J122" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="123" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A123" s="3" t="s">
         <v>138</v>
       </c>
@@ -4772,8 +6183,20 @@
       <c r="E123" s="5">
         <v>76.176000000000016</v>
       </c>
-    </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F123">
+        <v>15</v>
+      </c>
+      <c r="G123" t="s">
+        <v>12</v>
+      </c>
+      <c r="H123" t="s">
+        <v>15</v>
+      </c>
+      <c r="J123" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="124" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A124" s="3" t="s">
         <v>139</v>
       </c>
@@ -4789,8 +6212,20 @@
       <c r="E124" s="5">
         <v>76.176000000000016</v>
       </c>
-    </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F124">
+        <v>15</v>
+      </c>
+      <c r="G124" t="s">
+        <v>12</v>
+      </c>
+      <c r="H124" t="s">
+        <v>16</v>
+      </c>
+      <c r="J124" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="125" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A125" s="3" t="s">
         <v>140</v>
       </c>
@@ -4806,8 +6241,20 @@
       <c r="E125" s="5">
         <v>133.30799999999999</v>
       </c>
-    </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F125">
+        <v>15</v>
+      </c>
+      <c r="G125" t="s">
+        <v>671</v>
+      </c>
+      <c r="H125" t="s">
+        <v>11</v>
+      </c>
+      <c r="J125" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="126" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A126" s="3" t="s">
         <v>141</v>
       </c>
@@ -4823,8 +6270,20 @@
       <c r="E126" s="5">
         <v>76.176000000000016</v>
       </c>
-    </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F126">
+        <v>15</v>
+      </c>
+      <c r="G126" t="s">
+        <v>671</v>
+      </c>
+      <c r="H126" t="s">
+        <v>13</v>
+      </c>
+      <c r="J126" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="127" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A127" s="3" t="s">
         <v>142</v>
       </c>
@@ -4840,8 +6299,20 @@
       <c r="E127" s="5">
         <v>76.176000000000016</v>
       </c>
-    </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F127">
+        <v>15</v>
+      </c>
+      <c r="G127" t="s">
+        <v>671</v>
+      </c>
+      <c r="H127" t="s">
+        <v>14</v>
+      </c>
+      <c r="J127" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="128" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A128" s="3" t="s">
         <v>143</v>
       </c>
@@ -4857,8 +6328,20 @@
       <c r="E128" s="5">
         <v>76.176000000000016</v>
       </c>
-    </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F128">
+        <v>15</v>
+      </c>
+      <c r="G128" t="s">
+        <v>671</v>
+      </c>
+      <c r="H128" t="s">
+        <v>15</v>
+      </c>
+      <c r="J128" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="129" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A129" s="3" t="s">
         <v>144</v>
       </c>
@@ -4874,8 +6357,20 @@
       <c r="E129" s="5">
         <v>76.176000000000016</v>
       </c>
-    </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F129">
+        <v>15</v>
+      </c>
+      <c r="G129" t="s">
+        <v>671</v>
+      </c>
+      <c r="H129" t="s">
+        <v>16</v>
+      </c>
+      <c r="J129" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="130" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A130" s="3" t="s">
         <v>145</v>
       </c>
@@ -4891,8 +6386,20 @@
       <c r="E130" s="5">
         <v>76.176000000000016</v>
       </c>
-    </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F130">
+        <v>0</v>
+      </c>
+      <c r="G130" t="s">
+        <v>671</v>
+      </c>
+      <c r="H130" t="s">
+        <v>11</v>
+      </c>
+      <c r="J130" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="131" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A131" s="3" t="s">
         <v>146</v>
       </c>
@@ -4908,8 +6415,20 @@
       <c r="E131" s="5">
         <v>76.176000000000016</v>
       </c>
-    </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F131">
+        <v>10</v>
+      </c>
+      <c r="G131" t="s">
+        <v>671</v>
+      </c>
+      <c r="H131" t="s">
+        <v>13</v>
+      </c>
+      <c r="J131" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="132" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A132" s="3" t="s">
         <v>147</v>
       </c>
@@ -4925,8 +6444,20 @@
       <c r="E132" s="5">
         <v>76.176000000000016</v>
       </c>
-    </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F132">
+        <v>8</v>
+      </c>
+      <c r="G132" t="s">
+        <v>671</v>
+      </c>
+      <c r="H132" t="s">
+        <v>14</v>
+      </c>
+      <c r="J132" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="133" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A133" s="3" t="s">
         <v>148</v>
       </c>
@@ -4942,8 +6473,20 @@
       <c r="E133" s="5">
         <v>76.176000000000016</v>
       </c>
-    </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F133">
+        <v>5</v>
+      </c>
+      <c r="G133" t="s">
+        <v>671</v>
+      </c>
+      <c r="H133" t="s">
+        <v>15</v>
+      </c>
+      <c r="J133" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="134" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A134" s="3" t="s">
         <v>149</v>
       </c>
@@ -4959,8 +6502,20 @@
       <c r="E134" s="5">
         <v>76.176000000000016</v>
       </c>
-    </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F134">
+        <v>15</v>
+      </c>
+      <c r="G134" t="s">
+        <v>671</v>
+      </c>
+      <c r="H134" t="s">
+        <v>16</v>
+      </c>
+      <c r="J134" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="135" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A135" s="3" t="s">
         <v>150</v>
       </c>
@@ -4976,8 +6531,20 @@
       <c r="E135" s="5">
         <v>76.176000000000016</v>
       </c>
-    </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F135">
+        <v>15</v>
+      </c>
+      <c r="G135" t="s">
+        <v>671</v>
+      </c>
+      <c r="H135" t="s">
+        <v>11</v>
+      </c>
+      <c r="J135" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="136" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A136" s="3" t="s">
         <v>151</v>
       </c>
@@ -4993,8 +6560,20 @@
       <c r="E136" s="5">
         <v>142.83000000000001</v>
       </c>
-    </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F136">
+        <v>15</v>
+      </c>
+      <c r="G136" t="s">
+        <v>672</v>
+      </c>
+      <c r="H136" t="s">
+        <v>13</v>
+      </c>
+      <c r="J136" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="137" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A137" s="3" t="s">
         <v>152</v>
       </c>
@@ -5010,8 +6589,20 @@
       <c r="E137" s="5">
         <v>142.83000000000001</v>
       </c>
-    </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F137">
+        <v>15</v>
+      </c>
+      <c r="G137" t="s">
+        <v>672</v>
+      </c>
+      <c r="H137" t="s">
+        <v>14</v>
+      </c>
+      <c r="J137" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="138" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A138" s="3" t="s">
         <v>153</v>
       </c>
@@ -5027,8 +6618,20 @@
       <c r="E138" s="5">
         <v>142.83000000000001</v>
       </c>
-    </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F138">
+        <v>15</v>
+      </c>
+      <c r="G138" t="s">
+        <v>672</v>
+      </c>
+      <c r="H138" t="s">
+        <v>15</v>
+      </c>
+      <c r="J138" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="139" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A139" s="3" t="s">
         <v>154</v>
       </c>
@@ -5044,8 +6647,20 @@
       <c r="E139" s="5">
         <v>142.83000000000001</v>
       </c>
-    </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F139">
+        <v>15</v>
+      </c>
+      <c r="G139" t="s">
+        <v>672</v>
+      </c>
+      <c r="H139" t="s">
+        <v>16</v>
+      </c>
+      <c r="J139" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="140" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A140" s="3" t="s">
         <v>155</v>
       </c>
@@ -5061,8 +6676,20 @@
       <c r="E140" s="5">
         <v>142.83000000000001</v>
       </c>
-    </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F140">
+        <v>15</v>
+      </c>
+      <c r="G140" t="s">
+        <v>672</v>
+      </c>
+      <c r="H140" t="s">
+        <v>11</v>
+      </c>
+      <c r="J140" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="141" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A141" s="3" t="s">
         <v>156</v>
       </c>
@@ -5078,8 +6705,20 @@
       <c r="E141" s="5">
         <v>142.83000000000001</v>
       </c>
-    </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F141">
+        <v>15</v>
+      </c>
+      <c r="G141" t="s">
+        <v>672</v>
+      </c>
+      <c r="H141" t="s">
+        <v>13</v>
+      </c>
+      <c r="J141" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="142" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A142" s="3" t="s">
         <v>157</v>
       </c>
@@ -5095,8 +6734,20 @@
       <c r="E142" s="5">
         <v>142.83000000000001</v>
       </c>
-    </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F142">
+        <v>15</v>
+      </c>
+      <c r="G142" t="s">
+        <v>672</v>
+      </c>
+      <c r="H142" t="s">
+        <v>14</v>
+      </c>
+      <c r="J142" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="143" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A143" s="3" t="s">
         <v>158</v>
       </c>
@@ -5112,8 +6763,20 @@
       <c r="E143" s="5">
         <v>142.83000000000001</v>
       </c>
-    </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F143">
+        <v>15</v>
+      </c>
+      <c r="G143" t="s">
+        <v>672</v>
+      </c>
+      <c r="H143" t="s">
+        <v>15</v>
+      </c>
+      <c r="J143" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="144" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A144" s="3" t="s">
         <v>159</v>
       </c>
@@ -5129,8 +6792,20 @@
       <c r="E144" s="5">
         <v>76.176000000000016</v>
       </c>
-    </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F144">
+        <v>15</v>
+      </c>
+      <c r="G144" t="s">
+        <v>672</v>
+      </c>
+      <c r="H144" t="s">
+        <v>16</v>
+      </c>
+      <c r="J144" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="145" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A145" s="3" t="s">
         <v>160</v>
       </c>
@@ -5146,8 +6821,20 @@
       <c r="E145" s="5">
         <v>76.176000000000016</v>
       </c>
-    </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F145">
+        <v>15</v>
+      </c>
+      <c r="G145" t="s">
+        <v>672</v>
+      </c>
+      <c r="H145" t="s">
+        <v>15</v>
+      </c>
+      <c r="J145" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="146" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A146" s="3" t="s">
         <v>161</v>
       </c>
@@ -5163,8 +6850,20 @@
       <c r="E146" s="5">
         <v>142.83000000000001</v>
       </c>
-    </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F146">
+        <v>15</v>
+      </c>
+      <c r="G146" t="s">
+        <v>672</v>
+      </c>
+      <c r="H146" t="s">
+        <v>16</v>
+      </c>
+      <c r="J146" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="147" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A147" s="3" t="s">
         <v>162</v>
       </c>
@@ -5180,8 +6879,20 @@
       <c r="E147" s="5">
         <v>142.83000000000001</v>
       </c>
-    </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F147">
+        <v>15</v>
+      </c>
+      <c r="G147" t="s">
+        <v>673</v>
+      </c>
+      <c r="H147" t="s">
+        <v>11</v>
+      </c>
+      <c r="J147" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="148" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A148" s="3" t="s">
         <v>163</v>
       </c>
@@ -5197,8 +6908,20 @@
       <c r="E148" s="5">
         <v>142.83000000000001</v>
       </c>
-    </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F148">
+        <v>15</v>
+      </c>
+      <c r="G148" t="s">
+        <v>673</v>
+      </c>
+      <c r="H148" t="s">
+        <v>13</v>
+      </c>
+      <c r="J148" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="149" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A149" s="3" t="s">
         <v>164</v>
       </c>
@@ -5214,8 +6937,20 @@
       <c r="E149" s="5">
         <v>133.30799999999999</v>
       </c>
-    </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F149">
+        <v>15</v>
+      </c>
+      <c r="G149" t="s">
+        <v>673</v>
+      </c>
+      <c r="H149" t="s">
+        <v>14</v>
+      </c>
+      <c r="J149" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="150" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A150" s="3" t="s">
         <v>165</v>
       </c>
@@ -5231,8 +6966,20 @@
       <c r="E150" s="5">
         <v>142.83000000000001</v>
       </c>
-    </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F150">
+        <v>15</v>
+      </c>
+      <c r="G150" t="s">
+        <v>673</v>
+      </c>
+      <c r="H150" t="s">
+        <v>15</v>
+      </c>
+      <c r="J150" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="151" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A151" s="3" t="s">
         <v>166</v>
       </c>
@@ -5248,8 +6995,20 @@
       <c r="E151" s="5">
         <v>142.83000000000001</v>
       </c>
-    </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F151">
+        <v>15</v>
+      </c>
+      <c r="G151" t="s">
+        <v>673</v>
+      </c>
+      <c r="H151" t="s">
+        <v>16</v>
+      </c>
+      <c r="J151" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="152" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A152" s="3" t="s">
         <v>167</v>
       </c>
@@ -5265,8 +7024,20 @@
       <c r="E152" s="5">
         <v>257.35849999999999</v>
       </c>
-    </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F152">
+        <v>15</v>
+      </c>
+      <c r="G152" t="s">
+        <v>673</v>
+      </c>
+      <c r="H152" t="s">
+        <v>11</v>
+      </c>
+      <c r="J152" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="153" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A153" s="3" t="s">
         <v>168</v>
       </c>
@@ -5282,8 +7053,20 @@
       <c r="E153" s="5">
         <v>257.35849999999999</v>
       </c>
-    </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F153">
+        <v>15</v>
+      </c>
+      <c r="G153" t="s">
+        <v>673</v>
+      </c>
+      <c r="H153" t="s">
+        <v>13</v>
+      </c>
+      <c r="J153" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="154" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A154" s="3" t="s">
         <v>169</v>
       </c>
@@ -5299,8 +7082,20 @@
       <c r="E154" s="5">
         <v>257.35849999999999</v>
       </c>
-    </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F154">
+        <v>0</v>
+      </c>
+      <c r="G154" t="s">
+        <v>673</v>
+      </c>
+      <c r="H154" t="s">
+        <v>14</v>
+      </c>
+      <c r="J154" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="155" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A155" s="3" t="s">
         <v>170</v>
       </c>
@@ -5316,8 +7111,20 @@
       <c r="E155" s="5">
         <v>257.35849999999999</v>
       </c>
-    </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F155">
+        <v>10</v>
+      </c>
+      <c r="G155" t="s">
+        <v>673</v>
+      </c>
+      <c r="H155" t="s">
+        <v>15</v>
+      </c>
+      <c r="J155" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="156" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A156" s="3" t="s">
         <v>171</v>
       </c>
@@ -5333,8 +7140,20 @@
       <c r="E156" s="5">
         <v>76.176000000000016</v>
       </c>
-    </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F156">
+        <v>8</v>
+      </c>
+      <c r="G156" t="s">
+        <v>674</v>
+      </c>
+      <c r="H156" t="s">
+        <v>16</v>
+      </c>
+      <c r="J156" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="157" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A157" s="3" t="s">
         <v>172</v>
       </c>
@@ -5350,8 +7169,20 @@
       <c r="E157" s="5">
         <v>76.176000000000016</v>
       </c>
-    </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F157">
+        <v>5</v>
+      </c>
+      <c r="G157" t="s">
+        <v>674</v>
+      </c>
+      <c r="H157" t="s">
+        <v>11</v>
+      </c>
+      <c r="J157" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="158" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A158" s="3" t="s">
         <v>173</v>
       </c>
@@ -5367,8 +7198,20 @@
       <c r="E158" s="5">
         <v>171.39599999999999</v>
       </c>
-    </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F158">
+        <v>0</v>
+      </c>
+      <c r="G158" t="s">
+        <v>674</v>
+      </c>
+      <c r="H158" t="s">
+        <v>13</v>
+      </c>
+      <c r="J158" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="159" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A159" s="3" t="s">
         <v>174</v>
       </c>
@@ -5384,8 +7227,20 @@
       <c r="E159" s="5">
         <v>171.39599999999999</v>
       </c>
-    </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F159">
+        <v>10</v>
+      </c>
+      <c r="G159" t="s">
+        <v>674</v>
+      </c>
+      <c r="H159" t="s">
+        <v>14</v>
+      </c>
+      <c r="J159" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="160" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A160" s="3" t="s">
         <v>175</v>
       </c>
@@ -5401,8 +7256,20 @@
       <c r="E160" s="5">
         <v>171.39599999999999</v>
       </c>
-    </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F160">
+        <v>8</v>
+      </c>
+      <c r="G160" t="s">
+        <v>674</v>
+      </c>
+      <c r="H160" t="s">
+        <v>15</v>
+      </c>
+      <c r="J160" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="161" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A161" s="3" t="s">
         <v>176</v>
       </c>
@@ -5418,8 +7285,20 @@
       <c r="E161" s="5">
         <v>171.39599999999999</v>
       </c>
-    </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F161">
+        <v>5</v>
+      </c>
+      <c r="G161" t="s">
+        <v>674</v>
+      </c>
+      <c r="H161" t="s">
+        <v>16</v>
+      </c>
+      <c r="J161" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="162" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A162" s="3" t="s">
         <v>177</v>
       </c>
@@ -5435,8 +7314,20 @@
       <c r="E162" s="5">
         <v>171.39599999999999</v>
       </c>
-    </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F162">
+        <v>0</v>
+      </c>
+      <c r="G162" t="s">
+        <v>674</v>
+      </c>
+      <c r="H162" t="s">
+        <v>11</v>
+      </c>
+      <c r="J162" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="163" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A163" s="3" t="s">
         <v>178</v>
       </c>
@@ -5452,8 +7343,20 @@
       <c r="E163" s="5">
         <v>266.61599999999999</v>
       </c>
-    </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F163">
+        <v>10</v>
+      </c>
+      <c r="G163" t="s">
+        <v>674</v>
+      </c>
+      <c r="H163" t="s">
+        <v>13</v>
+      </c>
+      <c r="J163" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="164" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A164" s="3" t="s">
         <v>179</v>
       </c>
@@ -5469,8 +7372,20 @@
       <c r="E164" s="5">
         <v>266.61599999999999</v>
       </c>
-    </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F164">
+        <v>8</v>
+      </c>
+      <c r="G164" t="s">
+        <v>674</v>
+      </c>
+      <c r="H164" t="s">
+        <v>14</v>
+      </c>
+      <c r="J164" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="165" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A165" s="3" t="s">
         <v>180</v>
       </c>
@@ -5486,8 +7401,20 @@
       <c r="E165" s="5">
         <v>266.61599999999999</v>
       </c>
-    </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F165">
+        <v>5</v>
+      </c>
+      <c r="G165" t="s">
+        <v>675</v>
+      </c>
+      <c r="H165" t="s">
+        <v>15</v>
+      </c>
+      <c r="J165" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="166" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A166" s="3" t="s">
         <v>181</v>
       </c>
@@ -5503,8 +7430,20 @@
       <c r="E166" s="5">
         <v>266.61599999999999</v>
       </c>
-    </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F166">
+        <v>15</v>
+      </c>
+      <c r="G166" t="s">
+        <v>675</v>
+      </c>
+      <c r="H166" t="s">
+        <v>16</v>
+      </c>
+      <c r="J166" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="167" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A167" s="3" t="s">
         <v>182</v>
       </c>
@@ -5520,8 +7459,20 @@
       <c r="E167" s="5">
         <v>266.61599999999999</v>
       </c>
-    </row>
-    <row r="168" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F167">
+        <v>15</v>
+      </c>
+      <c r="G167" t="s">
+        <v>675</v>
+      </c>
+      <c r="H167" t="s">
+        <v>16</v>
+      </c>
+      <c r="J167" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="168" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A168" s="3" t="s">
         <v>183</v>
       </c>
@@ -5537,8 +7488,20 @@
       <c r="E168" s="5">
         <v>266.61599999999999</v>
       </c>
-    </row>
-    <row r="169" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F168">
+        <v>15</v>
+      </c>
+      <c r="G168" t="s">
+        <v>675</v>
+      </c>
+      <c r="H168" t="s">
+        <v>11</v>
+      </c>
+      <c r="J168" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="169" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A169" s="3" t="s">
         <v>184</v>
       </c>
@@ -5554,8 +7517,20 @@
       <c r="E169" s="5">
         <v>266.61599999999999</v>
       </c>
-    </row>
-    <row r="170" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F169">
+        <v>15</v>
+      </c>
+      <c r="G169" t="s">
+        <v>675</v>
+      </c>
+      <c r="H169" t="s">
+        <v>13</v>
+      </c>
+      <c r="J169" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="170" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A170" s="3" t="s">
         <v>185</v>
       </c>
@@ -5571,8 +7546,20 @@
       <c r="E170" s="5">
         <v>266.61599999999999</v>
       </c>
-    </row>
-    <row r="171" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F170">
+        <v>15</v>
+      </c>
+      <c r="G170" t="s">
+        <v>675</v>
+      </c>
+      <c r="H170" t="s">
+        <v>14</v>
+      </c>
+      <c r="J170" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="171" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A171" s="3" t="s">
         <v>186</v>
       </c>
@@ -5588,8 +7575,20 @@
       <c r="E171" s="5">
         <v>266.61599999999999</v>
       </c>
-    </row>
-    <row r="172" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F171">
+        <v>15</v>
+      </c>
+      <c r="G171" t="s">
+        <v>675</v>
+      </c>
+      <c r="H171" t="s">
+        <v>15</v>
+      </c>
+      <c r="J171" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="172" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A172" s="3" t="s">
         <v>187</v>
       </c>
@@ -5605,8 +7604,20 @@
       <c r="E172" s="5">
         <v>238.05</v>
       </c>
-    </row>
-    <row r="173" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F172">
+        <v>15</v>
+      </c>
+      <c r="G172" t="s">
+        <v>675</v>
+      </c>
+      <c r="H172" t="s">
+        <v>16</v>
+      </c>
+      <c r="J172" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="173" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A173" s="3" t="s">
         <v>188</v>
       </c>
@@ -5622,8 +7633,20 @@
       <c r="E173" s="5">
         <v>238.05</v>
       </c>
-    </row>
-    <row r="174" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F173">
+        <v>15</v>
+      </c>
+      <c r="G173" t="s">
+        <v>671</v>
+      </c>
+      <c r="H173" t="s">
+        <v>16</v>
+      </c>
+      <c r="J173" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="174" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A174" s="3" t="s">
         <v>189</v>
       </c>
@@ -5639,8 +7662,20 @@
       <c r="E174" s="5">
         <v>238.05</v>
       </c>
-    </row>
-    <row r="175" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F174">
+        <v>15</v>
+      </c>
+      <c r="G174" t="s">
+        <v>671</v>
+      </c>
+      <c r="H174" t="s">
+        <v>11</v>
+      </c>
+      <c r="J174" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="175" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A175" s="3" t="s">
         <v>190</v>
       </c>
@@ -5656,8 +7691,20 @@
       <c r="E175" s="5">
         <v>238.05</v>
       </c>
-    </row>
-    <row r="176" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F175">
+        <v>15</v>
+      </c>
+      <c r="G175" t="s">
+        <v>671</v>
+      </c>
+      <c r="H175" t="s">
+        <v>13</v>
+      </c>
+      <c r="J175" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="176" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A176" s="3" t="s">
         <v>191</v>
       </c>
@@ -5673,8 +7720,20 @@
       <c r="E176" s="5">
         <v>238.05</v>
       </c>
-    </row>
-    <row r="177" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F176">
+        <v>15</v>
+      </c>
+      <c r="G176" t="s">
+        <v>671</v>
+      </c>
+      <c r="H176" t="s">
+        <v>14</v>
+      </c>
+      <c r="J176" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="177" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A177" s="3" t="s">
         <v>192</v>
       </c>
@@ -5690,8 +7749,20 @@
       <c r="E177" s="5">
         <v>238.05</v>
       </c>
-    </row>
-    <row r="178" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F177">
+        <v>15</v>
+      </c>
+      <c r="G177" t="s">
+        <v>671</v>
+      </c>
+      <c r="H177" t="s">
+        <v>15</v>
+      </c>
+      <c r="J177" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="178" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A178" s="3" t="s">
         <v>193</v>
       </c>
@@ -5707,8 +7778,20 @@
       <c r="E178" s="5">
         <v>249.95249999999999</v>
       </c>
-    </row>
-    <row r="179" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F178">
+        <v>15</v>
+      </c>
+      <c r="G178" t="s">
+        <v>671</v>
+      </c>
+      <c r="H178" t="s">
+        <v>16</v>
+      </c>
+      <c r="J178" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="179" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A179" s="3" t="s">
         <v>194</v>
       </c>
@@ -5724,8 +7807,23 @@
       <c r="E179" s="5">
         <v>249.95249999999999</v>
       </c>
-    </row>
-    <row r="180" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F179">
+        <v>15</v>
+      </c>
+      <c r="G179" t="s">
+        <v>12</v>
+      </c>
+      <c r="H179" t="s">
+        <v>11</v>
+      </c>
+      <c r="I179" t="s">
+        <v>10</v>
+      </c>
+      <c r="J179" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="180" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A180" s="3" t="s">
         <v>195</v>
       </c>
@@ -5741,8 +7839,20 @@
       <c r="E180" s="5">
         <v>249.95249999999999</v>
       </c>
-    </row>
-    <row r="181" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F180">
+        <v>0</v>
+      </c>
+      <c r="G180" t="s">
+        <v>12</v>
+      </c>
+      <c r="H180" t="s">
+        <v>13</v>
+      </c>
+      <c r="J180" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="181" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A181" s="3" t="s">
         <v>196</v>
       </c>
@@ -5758,8 +7868,20 @@
       <c r="E181" s="5">
         <v>75.382499999999993</v>
       </c>
-    </row>
-    <row r="182" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F181">
+        <v>10</v>
+      </c>
+      <c r="G181" t="s">
+        <v>12</v>
+      </c>
+      <c r="H181" t="s">
+        <v>14</v>
+      </c>
+      <c r="J181" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="182" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A182" s="3" t="s">
         <v>197</v>
       </c>
@@ -5775,8 +7897,20 @@
       <c r="E182" s="5">
         <v>92.575000000000003</v>
       </c>
-    </row>
-    <row r="183" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F182">
+        <v>8</v>
+      </c>
+      <c r="G182" t="s">
+        <v>12</v>
+      </c>
+      <c r="H182" t="s">
+        <v>15</v>
+      </c>
+      <c r="J182" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="183" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A183" s="3" t="s">
         <v>198</v>
       </c>
@@ -5792,8 +7926,20 @@
       <c r="E183" s="5">
         <v>128.2825</v>
       </c>
-    </row>
-    <row r="184" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F183">
+        <v>5</v>
+      </c>
+      <c r="G183" t="s">
+        <v>12</v>
+      </c>
+      <c r="H183" t="s">
+        <v>16</v>
+      </c>
+      <c r="J183" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="184" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A184" s="3" t="s">
         <v>199</v>
       </c>
@@ -5809,8 +7955,20 @@
       <c r="E184" s="5">
         <v>74.06</v>
       </c>
-    </row>
-    <row r="185" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F184">
+        <v>15</v>
+      </c>
+      <c r="G184" t="s">
+        <v>671</v>
+      </c>
+      <c r="H184" t="s">
+        <v>11</v>
+      </c>
+      <c r="J184" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="185" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A185" s="3" t="s">
         <v>200</v>
       </c>
@@ -5826,8 +7984,20 @@
       <c r="E185" s="5">
         <v>2869.8249999999998</v>
       </c>
-    </row>
-    <row r="186" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F185">
+        <v>15</v>
+      </c>
+      <c r="G185" t="s">
+        <v>671</v>
+      </c>
+      <c r="H185" t="s">
+        <v>13</v>
+      </c>
+      <c r="J185" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="186" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A186" s="3" t="s">
         <v>201</v>
       </c>
@@ -5843,8 +8013,20 @@
       <c r="E186" s="5">
         <v>2406.9499999999998</v>
       </c>
-    </row>
-    <row r="187" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F186">
+        <v>15</v>
+      </c>
+      <c r="G186" t="s">
+        <v>671</v>
+      </c>
+      <c r="H186" t="s">
+        <v>14</v>
+      </c>
+      <c r="J186" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="187" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A187" s="3" t="s">
         <v>202</v>
       </c>
@@ -5860,8 +8042,20 @@
       <c r="E187" s="5">
         <v>2869.8249999999998</v>
       </c>
-    </row>
-    <row r="188" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F187">
+        <v>15</v>
+      </c>
+      <c r="G187" t="s">
+        <v>671</v>
+      </c>
+      <c r="H187" t="s">
+        <v>15</v>
+      </c>
+      <c r="J187" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="188" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A188" s="3" t="s">
         <v>203</v>
       </c>
@@ -5877,8 +8071,20 @@
       <c r="E188" s="5">
         <v>1454.75</v>
       </c>
-    </row>
-    <row r="189" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F188">
+        <v>15</v>
+      </c>
+      <c r="G188" t="s">
+        <v>671</v>
+      </c>
+      <c r="H188" t="s">
+        <v>16</v>
+      </c>
+      <c r="J188" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="189" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A189" s="3" t="s">
         <v>204</v>
       </c>
@@ -5894,8 +8100,20 @@
       <c r="E189" s="5">
         <v>1758.925</v>
       </c>
-    </row>
-    <row r="190" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F189">
+        <v>15</v>
+      </c>
+      <c r="G189" t="s">
+        <v>671</v>
+      </c>
+      <c r="H189" t="s">
+        <v>11</v>
+      </c>
+      <c r="J189" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="190" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A190" s="3" t="s">
         <v>205</v>
       </c>
@@ -5911,8 +8129,20 @@
       <c r="E190" s="5">
         <v>203.66499999999999</v>
       </c>
-    </row>
-    <row r="191" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F190">
+        <v>15</v>
+      </c>
+      <c r="G190" t="s">
+        <v>671</v>
+      </c>
+      <c r="H190" t="s">
+        <v>13</v>
+      </c>
+      <c r="J190" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="191" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A191" s="3" t="s">
         <v>206</v>
       </c>
@@ -5928,8 +8158,20 @@
       <c r="E191" s="5">
         <v>222.17999999999998</v>
       </c>
-    </row>
-    <row r="192" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F191">
+        <v>15</v>
+      </c>
+      <c r="G191" t="s">
+        <v>671</v>
+      </c>
+      <c r="H191" t="s">
+        <v>14</v>
+      </c>
+      <c r="J191" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="192" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A192" s="3" t="s">
         <v>207</v>
       </c>
@@ -5945,8 +8187,20 @@
       <c r="E192" s="5">
         <v>204.98750000000001</v>
       </c>
-    </row>
-    <row r="193" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F192">
+        <v>15</v>
+      </c>
+      <c r="G192" t="s">
+        <v>671</v>
+      </c>
+      <c r="H192" t="s">
+        <v>15</v>
+      </c>
+      <c r="J192" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="193" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A193" s="3" t="s">
         <v>208</v>
       </c>
@@ -5962,8 +8216,20 @@
       <c r="E193" s="5">
         <v>1758.925</v>
       </c>
-    </row>
-    <row r="194" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F193">
+        <v>0</v>
+      </c>
+      <c r="G193" t="s">
+        <v>671</v>
+      </c>
+      <c r="H193" t="s">
+        <v>16</v>
+      </c>
+      <c r="J193" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="194" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A194" s="3" t="s">
         <v>209</v>
       </c>
@@ -5979,8 +8245,20 @@
       <c r="E194" s="5">
         <v>1110.9000000000001</v>
       </c>
-    </row>
-    <row r="195" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F194">
+        <v>10</v>
+      </c>
+      <c r="G194" t="s">
+        <v>671</v>
+      </c>
+      <c r="H194" t="s">
+        <v>11</v>
+      </c>
+      <c r="J194" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="195" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A195" s="3" t="s">
         <v>210</v>
       </c>
@@ -5996,8 +8274,20 @@
       <c r="E195" s="5">
         <v>1758.925</v>
       </c>
-    </row>
-    <row r="196" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F195">
+        <v>8</v>
+      </c>
+      <c r="G195" t="s">
+        <v>672</v>
+      </c>
+      <c r="H195" t="s">
+        <v>13</v>
+      </c>
+      <c r="J195" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="196" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A196" s="3" t="s">
         <v>211</v>
       </c>
@@ -6013,8 +8303,20 @@
       <c r="E196" s="5">
         <v>1203.4749999999999</v>
       </c>
-    </row>
-    <row r="197" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F196">
+        <v>5</v>
+      </c>
+      <c r="G196" t="s">
+        <v>672</v>
+      </c>
+      <c r="H196" t="s">
+        <v>14</v>
+      </c>
+      <c r="J196" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="197" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A197" s="3" t="s">
         <v>212</v>
       </c>
@@ -6030,8 +8332,20 @@
       <c r="E197" s="5">
         <v>211.6</v>
       </c>
-    </row>
-    <row r="198" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F197">
+        <v>15</v>
+      </c>
+      <c r="G197" t="s">
+        <v>672</v>
+      </c>
+      <c r="H197" t="s">
+        <v>15</v>
+      </c>
+      <c r="J197" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="198" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A198" s="3" t="s">
         <v>213</v>
       </c>
@@ -6047,8 +8361,20 @@
       <c r="E198" s="5">
         <v>264.5</v>
       </c>
-    </row>
-    <row r="199" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F198">
+        <v>15</v>
+      </c>
+      <c r="G198" t="s">
+        <v>672</v>
+      </c>
+      <c r="H198" t="s">
+        <v>16</v>
+      </c>
+      <c r="J198" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="199" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A199" s="3" t="s">
         <v>214</v>
       </c>
@@ -6064,8 +8390,20 @@
       <c r="E199" s="5">
         <v>529</v>
       </c>
-    </row>
-    <row r="200" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F199">
+        <v>15</v>
+      </c>
+      <c r="G199" t="s">
+        <v>672</v>
+      </c>
+      <c r="H199" t="s">
+        <v>11</v>
+      </c>
+      <c r="J199" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="200" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A200" s="3" t="s">
         <v>215</v>
       </c>
@@ -6081,8 +8419,20 @@
       <c r="E200" s="5">
         <v>529</v>
       </c>
-    </row>
-    <row r="201" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F200">
+        <v>15</v>
+      </c>
+      <c r="G200" t="s">
+        <v>672</v>
+      </c>
+      <c r="H200" t="s">
+        <v>13</v>
+      </c>
+      <c r="J200" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="201" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A201" s="3" t="s">
         <v>216</v>
       </c>
@@ -6098,8 +8448,20 @@
       <c r="E201" s="5">
         <v>767.05</v>
       </c>
-    </row>
-    <row r="202" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F201">
+        <v>15</v>
+      </c>
+      <c r="G201" t="s">
+        <v>672</v>
+      </c>
+      <c r="H201" t="s">
+        <v>14</v>
+      </c>
+      <c r="J201" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="202" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A202" s="3" t="s">
         <v>217</v>
       </c>
@@ -6115,8 +8477,20 @@
       <c r="E202" s="5">
         <v>112.41249999999999</v>
       </c>
-    </row>
-    <row r="203" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F202">
+        <v>15</v>
+      </c>
+      <c r="G202" t="s">
+        <v>672</v>
+      </c>
+      <c r="H202" t="s">
+        <v>15</v>
+      </c>
+      <c r="J202" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="203" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A203" s="3" t="s">
         <v>218</v>
       </c>
@@ -6132,8 +8506,20 @@
       <c r="E203" s="5">
         <v>1785.375</v>
       </c>
-    </row>
-    <row r="204" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F203">
+        <v>15</v>
+      </c>
+      <c r="G203" t="s">
+        <v>672</v>
+      </c>
+      <c r="H203" t="s">
+        <v>16</v>
+      </c>
+      <c r="J203" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="204" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A204" s="3" t="s">
         <v>219</v>
       </c>
@@ -6149,8 +8535,20 @@
       <c r="E204" s="5">
         <v>101.8325</v>
       </c>
-    </row>
-    <row r="205" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F204">
+        <v>15</v>
+      </c>
+      <c r="G204" t="s">
+        <v>672</v>
+      </c>
+      <c r="H204" t="s">
+        <v>15</v>
+      </c>
+      <c r="J204" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="205" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A205" s="3" t="s">
         <v>220</v>
       </c>
@@ -6166,8 +8564,20 @@
       <c r="E205" s="5">
         <v>101.8325</v>
       </c>
-    </row>
-    <row r="206" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F205">
+        <v>15</v>
+      </c>
+      <c r="G205" t="s">
+        <v>672</v>
+      </c>
+      <c r="H205" t="s">
+        <v>16</v>
+      </c>
+      <c r="J205" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="206" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A206" s="3" t="s">
         <v>221</v>
       </c>
@@ -6183,8 +8593,20 @@
       <c r="E206" s="5">
         <v>101.8325</v>
       </c>
-    </row>
-    <row r="207" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F206">
+        <v>15</v>
+      </c>
+      <c r="G206" t="s">
+        <v>673</v>
+      </c>
+      <c r="H206" t="s">
+        <v>11</v>
+      </c>
+      <c r="J206" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="207" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A207" s="3" t="s">
         <v>222</v>
       </c>
@@ -6200,8 +8622,20 @@
       <c r="E207" s="5">
         <v>101.8325</v>
       </c>
-    </row>
-    <row r="208" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F207">
+        <v>15</v>
+      </c>
+      <c r="G207" t="s">
+        <v>673</v>
+      </c>
+      <c r="H207" t="s">
+        <v>13</v>
+      </c>
+      <c r="J207" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="208" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A208" s="3" t="s">
         <v>223</v>
       </c>
@@ -6217,8 +8651,20 @@
       <c r="E208" s="5">
         <v>284.33749999999998</v>
       </c>
-    </row>
-    <row r="209" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F208">
+        <v>15</v>
+      </c>
+      <c r="G208" t="s">
+        <v>673</v>
+      </c>
+      <c r="H208" t="s">
+        <v>14</v>
+      </c>
+      <c r="J208" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="209" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A209" s="3" t="s">
         <v>224</v>
       </c>
@@ -6234,8 +8680,20 @@
       <c r="E209" s="5">
         <v>284.33749999999998</v>
       </c>
-    </row>
-    <row r="210" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F209">
+        <v>15</v>
+      </c>
+      <c r="G209" t="s">
+        <v>673</v>
+      </c>
+      <c r="H209" t="s">
+        <v>15</v>
+      </c>
+      <c r="J209" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="210" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A210" s="3" t="s">
         <v>225</v>
       </c>
@@ -6251,8 +8709,20 @@
       <c r="E210" s="5">
         <v>284.33749999999998</v>
       </c>
-    </row>
-    <row r="211" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F210">
+        <v>15</v>
+      </c>
+      <c r="G210" t="s">
+        <v>673</v>
+      </c>
+      <c r="H210" t="s">
+        <v>16</v>
+      </c>
+      <c r="J210" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="211" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A211" s="3" t="s">
         <v>226</v>
       </c>
@@ -6268,8 +8738,20 @@
       <c r="E211" s="5">
         <v>284.33749999999998</v>
       </c>
-    </row>
-    <row r="212" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F211">
+        <v>15</v>
+      </c>
+      <c r="G211" t="s">
+        <v>673</v>
+      </c>
+      <c r="H211" t="s">
+        <v>11</v>
+      </c>
+      <c r="J211" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="212" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A212" s="3" t="s">
         <v>227</v>
       </c>
@@ -6285,8 +8767,20 @@
       <c r="E212" s="5">
         <v>373.60624999999999</v>
       </c>
-    </row>
-    <row r="213" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F212">
+        <v>15</v>
+      </c>
+      <c r="G212" t="s">
+        <v>673</v>
+      </c>
+      <c r="H212" t="s">
+        <v>13</v>
+      </c>
+      <c r="J212" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="213" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A213" s="3" t="s">
         <v>228</v>
       </c>
@@ -6302,8 +8796,20 @@
       <c r="E213" s="5">
         <v>396.75</v>
       </c>
-    </row>
-    <row r="221" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F213">
+        <v>15</v>
+      </c>
+      <c r="G213" t="s">
+        <v>673</v>
+      </c>
+      <c r="H213" t="s">
+        <v>14</v>
+      </c>
+      <c r="J213" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="221" spans="1:10" x14ac:dyDescent="0.3">
       <c r="B221"/>
     </row>
     <row r="227" spans="2:2" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
fix bulk upload V codex
</commit_message>
<xml_diff>
--- a/trial 1(AutoRecovered).xlsx
+++ b/trial 1(AutoRecovered).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\mohamed adel work\cesar-store\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2334EF8-B211-4783-A7C4-F575143A8387}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2DFC1CD-C7DE-4EB3-98C6-4F0F51719760}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{791D22A4-40A8-4DDB-9123-A17DB6BCCBDF}"/>
   </bookViews>
@@ -2585,18 +2585,12 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -2621,7 +2615,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -3082,7 +3076,7 @@
     <col min="4" max="4" width="36.44140625" customWidth="1"/>
     <col min="5" max="5" width="9.21875" customWidth="1"/>
     <col min="6" max="6" width="5.33203125" customWidth="1"/>
-    <col min="7" max="7" width="15.109375" customWidth="1"/>
+    <col min="7" max="7" width="15.109375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="30.6640625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="5.88671875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="6" bestFit="1" customWidth="1"/>

</xml_diff>